<commit_message>
Jcalc list: add 7401-7417 (NGA-East with S20/H20 and RS24 adjustments)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012hqFBNE5nDByFb9nHZs7cc
</commit_message>
<xml_diff>
--- a/docs/HAZ-45.4 Jcalc List.xlsx
+++ b/docs/HAZ-45.4 Jcalc List.xlsx
@@ -569,7 +569,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J332"/>
+  <dimension ref="A1:J350"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="10.75" defaultRowHeight="15.5"/>
   <cols>
     <col width="9.25" customWidth="1" style="15" min="1" max="1"/>
@@ -598,7 +598,6 @@
       <c r="C2" s="19" t="n"/>
       <c r="D2" s="19" t="n"/>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="B4" s="1" t="inlineStr">
         <is>
@@ -7030,22 +7029,50 @@
         </is>
       </c>
     </row>
-    <row r="272"/>
+    <row r="272">
+      <c r="B272" s="26" t="inlineStr">
+        <is>
+          <t>PEER NGA-East Ground Motion Models with Stewart et al. (2020) and Hashash et al. (2020) Site Amplification and Ramos-Sepulveda et al. (2024) Adjustments</t>
+        </is>
+      </c>
+    </row>
     <row r="273">
-      <c r="B273" s="26" t="inlineStr">
-        <is>
-          <t>NGA-Subduction</t>
+      <c r="B273" s="19" t="n">
+        <v>7401</v>
+      </c>
+      <c r="C273" s="22" t="n">
+        <v>25</v>
+      </c>
+      <c r="D273" s="23" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="E273" s="23" t="n">
+        <v>10</v>
+      </c>
+      <c r="F273" s="23" t="inlineStr">
+        <is>
+          <t>S34_NGAEast_Med, S34_NGAEast_SiteAmp, S34_NGAEast_RS24Adj</t>
+        </is>
+      </c>
+      <c r="G273" s="15" t="inlineStr">
+        <is>
+          <t>NGA-East 2018 Median Model No. 1 with Stewart et al. (2020) and Hashash et al. (2020) site amplification and Ramos-Sepulveda et al. (2024) adjustments</t>
+        </is>
+      </c>
+      <c r="H273" t="inlineStr">
+        <is>
+          <t>Median only; use with a sigma model (e.g., 7101-7106). VS30 must be 200-3000 m/s</t>
         </is>
       </c>
     </row>
     <row r="274">
-      <c r="B274" s="22" t="n">
-        <v>390</v>
+      <c r="B274" s="19" t="n">
+        <v>7402</v>
       </c>
       <c r="C274" s="22" t="n">
         <v>25</v>
       </c>
-      <c r="D274" s="22" t="n">
+      <c r="D274" s="23" t="n">
         <v>0.01</v>
       </c>
       <c r="E274" s="23" t="n">
@@ -7053,23 +7080,28 @@
       </c>
       <c r="F274" s="23" t="inlineStr">
         <is>
-          <t>S35_AG2020</t>
+          <t>S34_NGAEast_Med, S34_NGAEast_SiteAmp, S34_NGAEast_RS24Adj</t>
         </is>
       </c>
       <c r="G274" s="15" t="inlineStr">
         <is>
-          <t>Abrahamson&amp;Gulerce (2020), Alaska without adjustments</t>
+          <t>NGA-East 2018 Median Model No. 2 with Stewart et al. (2020) and Hashash et al. (2020) site amplification and Ramos-Sepulveda et al. (2024) adjustments</t>
+        </is>
+      </c>
+      <c r="H274" t="inlineStr">
+        <is>
+          <t>Median only; use with a sigma model (e.g., 7101-7106). VS30 must be 200-3000 m/s</t>
         </is>
       </c>
     </row>
     <row r="275">
-      <c r="B275" s="22" t="n">
-        <v>391</v>
+      <c r="B275" s="19" t="n">
+        <v>7403</v>
       </c>
       <c r="C275" s="22" t="n">
         <v>25</v>
       </c>
-      <c r="D275" s="22" t="n">
+      <c r="D275" s="23" t="n">
         <v>0.01</v>
       </c>
       <c r="E275" s="23" t="n">
@@ -7077,23 +7109,28 @@
       </c>
       <c r="F275" s="23" t="inlineStr">
         <is>
-          <t>S35_AG2020</t>
+          <t>S34_NGAEast_Med, S34_NGAEast_SiteAmp, S34_NGAEast_RS24Adj</t>
         </is>
       </c>
       <c r="G275" s="15" t="inlineStr">
         <is>
-          <t>Abrahamson&amp;Gulerce (2020), Alaska with adjustments</t>
+          <t>NGA-East 2018 Median Model No. 3 with Stewart et al. (2020) and Hashash et al. (2020) site amplification and Ramos-Sepulveda et al. (2024) adjustments</t>
+        </is>
+      </c>
+      <c r="H275" t="inlineStr">
+        <is>
+          <t>Median only; use with a sigma model (e.g., 7101-7106). VS30 must be 200-3000 m/s</t>
         </is>
       </c>
     </row>
     <row r="276">
-      <c r="B276" s="22" t="n">
-        <v>392</v>
+      <c r="B276" s="19" t="n">
+        <v>7404</v>
       </c>
       <c r="C276" s="22" t="n">
         <v>25</v>
       </c>
-      <c r="D276" s="22" t="n">
+      <c r="D276" s="23" t="n">
         <v>0.01</v>
       </c>
       <c r="E276" s="23" t="n">
@@ -7101,23 +7138,28 @@
       </c>
       <c r="F276" s="23" t="inlineStr">
         <is>
-          <t>S35_AG2020</t>
+          <t>S34_NGAEast_Med, S34_NGAEast_SiteAmp, S34_NGAEast_RS24Adj</t>
         </is>
       </c>
       <c r="G276" s="15" t="inlineStr">
         <is>
-          <t>Abrahamson&amp;Gulerce (2020), Cascadia with adjustments</t>
+          <t>NGA-East 2018 Median Model No. 4 with Stewart et al. (2020) and Hashash et al. (2020) site amplification and Ramos-Sepulveda et al. (2024) adjustments</t>
+        </is>
+      </c>
+      <c r="H276" t="inlineStr">
+        <is>
+          <t>Median only; use with a sigma model (e.g., 7101-7106). VS30 must be 200-3000 m/s</t>
         </is>
       </c>
     </row>
     <row r="277">
-      <c r="B277" s="22" t="n">
-        <v>393</v>
+      <c r="B277" s="19" t="n">
+        <v>7405</v>
       </c>
       <c r="C277" s="22" t="n">
         <v>25</v>
       </c>
-      <c r="D277" s="22" t="n">
+      <c r="D277" s="23" t="n">
         <v>0.01</v>
       </c>
       <c r="E277" s="23" t="n">
@@ -7125,23 +7167,28 @@
       </c>
       <c r="F277" s="23" t="inlineStr">
         <is>
-          <t>S35_AG2020</t>
+          <t>S34_NGAEast_Med, S34_NGAEast_SiteAmp, S34_NGAEast_RS24Adj</t>
         </is>
       </c>
       <c r="G277" s="15" t="inlineStr">
         <is>
-          <t>Abrahamson&amp;Gulerce (2020), Central Am/Mexico</t>
+          <t>NGA-East 2018 Median Model No. 5 with Stewart et al. (2020) and Hashash et al. (2020) site amplification and Ramos-Sepulveda et al. (2024) adjustments</t>
+        </is>
+      </c>
+      <c r="H277" t="inlineStr">
+        <is>
+          <t>Median only; use with a sigma model (e.g., 7101-7106). VS30 must be 200-3000 m/s</t>
         </is>
       </c>
     </row>
     <row r="278">
-      <c r="B278" s="22" t="n">
-        <v>394</v>
+      <c r="B278" s="19" t="n">
+        <v>7406</v>
       </c>
       <c r="C278" s="22" t="n">
         <v>25</v>
       </c>
-      <c r="D278" s="22" t="n">
+      <c r="D278" s="23" t="n">
         <v>0.01</v>
       </c>
       <c r="E278" s="23" t="n">
@@ -7149,23 +7196,28 @@
       </c>
       <c r="F278" s="23" t="inlineStr">
         <is>
-          <t>S35_AG2020</t>
+          <t>S34_NGAEast_Med, S34_NGAEast_SiteAmp, S34_NGAEast_RS24Adj</t>
         </is>
       </c>
       <c r="G278" s="15" t="inlineStr">
         <is>
-          <t>Abrahamson&amp;Gulerce (2020), Japan</t>
+          <t>NGA-East 2018 Median Model No. 6 with Stewart et al. (2020) and Hashash et al. (2020) site amplification and Ramos-Sepulveda et al. (2024) adjustments</t>
+        </is>
+      </c>
+      <c r="H278" t="inlineStr">
+        <is>
+          <t>Median only; use with a sigma model (e.g., 7101-7106). VS30 must be 200-3000 m/s</t>
         </is>
       </c>
     </row>
     <row r="279">
-      <c r="B279" s="22" t="n">
-        <v>395</v>
+      <c r="B279" s="19" t="n">
+        <v>7407</v>
       </c>
       <c r="C279" s="22" t="n">
         <v>25</v>
       </c>
-      <c r="D279" s="22" t="n">
+      <c r="D279" s="23" t="n">
         <v>0.01</v>
       </c>
       <c r="E279" s="23" t="n">
@@ -7173,23 +7225,28 @@
       </c>
       <c r="F279" s="23" t="inlineStr">
         <is>
-          <t>S35_AG2020</t>
+          <t>S34_NGAEast_Med, S34_NGAEast_SiteAmp, S34_NGAEast_RS24Adj</t>
         </is>
       </c>
       <c r="G279" s="15" t="inlineStr">
         <is>
-          <t>Abrahamson&amp;Gulerce (2020), New Zealand</t>
+          <t>NGA-East 2018 Median Model No. 7 with Stewart et al. (2020) and Hashash et al. (2020) site amplification and Ramos-Sepulveda et al. (2024) adjustments</t>
+        </is>
+      </c>
+      <c r="H279" t="inlineStr">
+        <is>
+          <t>Median only; use with a sigma model (e.g., 7101-7106). VS30 must be 200-3000 m/s</t>
         </is>
       </c>
     </row>
     <row r="280">
-      <c r="B280" s="22" t="n">
-        <v>396</v>
+      <c r="B280" s="19" t="n">
+        <v>7408</v>
       </c>
       <c r="C280" s="22" t="n">
         <v>25</v>
       </c>
-      <c r="D280" s="22" t="n">
+      <c r="D280" s="23" t="n">
         <v>0.01</v>
       </c>
       <c r="E280" s="23" t="n">
@@ -7197,23 +7254,28 @@
       </c>
       <c r="F280" s="23" t="inlineStr">
         <is>
-          <t>S35_AG2020</t>
+          <t>S34_NGAEast_Med, S34_NGAEast_SiteAmp, S34_NGAEast_RS24Adj</t>
         </is>
       </c>
       <c r="G280" s="15" t="inlineStr">
         <is>
-          <t>Abrahamson&amp;Gulerce (2020), South America</t>
+          <t>NGA-East 2018 Median Model No. 8 with Stewart et al. (2020) and Hashash et al. (2020) site amplification and Ramos-Sepulveda et al. (2024) adjustments</t>
+        </is>
+      </c>
+      <c r="H280" t="inlineStr">
+        <is>
+          <t>Median only; use with a sigma model (e.g., 7101-7106). VS30 must be 200-3000 m/s</t>
         </is>
       </c>
     </row>
     <row r="281">
-      <c r="B281" s="22" t="n">
-        <v>397</v>
+      <c r="B281" s="19" t="n">
+        <v>7409</v>
       </c>
       <c r="C281" s="22" t="n">
         <v>25</v>
       </c>
-      <c r="D281" s="22" t="n">
+      <c r="D281" s="23" t="n">
         <v>0.01</v>
       </c>
       <c r="E281" s="23" t="n">
@@ -7221,23 +7283,28 @@
       </c>
       <c r="F281" s="23" t="inlineStr">
         <is>
-          <t>S35_AG2020</t>
+          <t>S34_NGAEast_Med, S34_NGAEast_SiteAmp, S34_NGAEast_RS24Adj</t>
         </is>
       </c>
       <c r="G281" s="15" t="inlineStr">
         <is>
-          <t>Abrahamson&amp;Gulerce (2020), Taiwan</t>
+          <t>NGA-East 2018 Median Model No. 9 with Stewart et al. (2020) and Hashash et al. (2020) site amplification and Ramos-Sepulveda et al. (2024) adjustments</t>
+        </is>
+      </c>
+      <c r="H281" t="inlineStr">
+        <is>
+          <t>Median only; use with a sigma model (e.g., 7101-7106). VS30 must be 200-3000 m/s</t>
         </is>
       </c>
     </row>
     <row r="282">
-      <c r="B282" s="22" t="n">
-        <v>398</v>
+      <c r="B282" s="19" t="n">
+        <v>7410</v>
       </c>
       <c r="C282" s="22" t="n">
         <v>25</v>
       </c>
-      <c r="D282" s="22" t="n">
+      <c r="D282" s="23" t="n">
         <v>0.01</v>
       </c>
       <c r="E282" s="23" t="n">
@@ -7245,23 +7312,28 @@
       </c>
       <c r="F282" s="23" t="inlineStr">
         <is>
-          <t>S35_AG2020</t>
+          <t>S34_NGAEast_Med, S34_NGAEast_SiteAmp, S34_NGAEast_RS24Adj</t>
         </is>
       </c>
       <c r="G282" s="15" t="inlineStr">
         <is>
-          <t>Abrahamson&amp;Gulerce (2020), Global</t>
+          <t>NGA-East 2018 Median Model No. 10 with Stewart et al. (2020) and Hashash et al. (2020) site amplification and Ramos-Sepulveda et al. (2024) adjustments</t>
+        </is>
+      </c>
+      <c r="H282" t="inlineStr">
+        <is>
+          <t>Median only; use with a sigma model (e.g., 7101-7106). VS30 must be 200-3000 m/s</t>
         </is>
       </c>
     </row>
     <row r="283">
-      <c r="B283" s="22" t="n">
-        <v>399</v>
+      <c r="B283" s="19" t="n">
+        <v>7411</v>
       </c>
       <c r="C283" s="22" t="n">
         <v>25</v>
       </c>
-      <c r="D283" s="22" t="n">
+      <c r="D283" s="23" t="n">
         <v>0.01</v>
       </c>
       <c r="E283" s="23" t="n">
@@ -7269,23 +7341,28 @@
       </c>
       <c r="F283" s="23" t="inlineStr">
         <is>
-          <t>S35_AG2020</t>
+          <t>S34_NGAEast_Med, S34_NGAEast_SiteAmp, S34_NGAEast_RS24Adj</t>
         </is>
       </c>
       <c r="G283" s="15" t="inlineStr">
         <is>
-          <t>Abrahamson&amp;Gulerce (2020), Cascadia without adjustments</t>
+          <t>NGA-East 2018 Median Model No. 11 with Stewart et al. (2020) and Hashash et al. (2020) site amplification and Ramos-Sepulveda et al. (2024) adjustments</t>
+        </is>
+      </c>
+      <c r="H283" t="inlineStr">
+        <is>
+          <t>Median only; use with a sigma model (e.g., 7101-7106). VS30 must be 200-3000 m/s</t>
         </is>
       </c>
     </row>
     <row r="284">
-      <c r="B284" s="22" t="n">
-        <v>1398</v>
+      <c r="B284" s="19" t="n">
+        <v>7412</v>
       </c>
       <c r="C284" s="22" t="n">
         <v>25</v>
       </c>
-      <c r="D284" s="22" t="n">
+      <c r="D284" s="23" t="n">
         <v>0.01</v>
       </c>
       <c r="E284" s="23" t="n">
@@ -7293,23 +7370,28 @@
       </c>
       <c r="F284" s="23" t="inlineStr">
         <is>
-          <t>S35_AG2020</t>
+          <t>S34_NGAEast_Med, S34_NGAEast_SiteAmp, S34_NGAEast_RS24Adj</t>
         </is>
       </c>
       <c r="G284" s="15" t="inlineStr">
         <is>
-          <t>Abrahamson&amp;Gulerce (2020), Global lower Epistemic Model</t>
+          <t>NGA-East 2018 Median Model No. 12 with Stewart et al. (2020) and Hashash et al. (2020) site amplification and Ramos-Sepulveda et al. (2024) adjustments</t>
+        </is>
+      </c>
+      <c r="H284" t="inlineStr">
+        <is>
+          <t>Median only; use with a sigma model (e.g., 7101-7106). VS30 must be 200-3000 m/s</t>
         </is>
       </c>
     </row>
     <row r="285">
-      <c r="B285" s="22" t="n">
-        <v>2398</v>
+      <c r="B285" s="19" t="n">
+        <v>7413</v>
       </c>
       <c r="C285" s="22" t="n">
         <v>25</v>
       </c>
-      <c r="D285" s="22" t="n">
+      <c r="D285" s="23" t="n">
         <v>0.01</v>
       </c>
       <c r="E285" s="23" t="n">
@@ -7317,23 +7399,28 @@
       </c>
       <c r="F285" s="23" t="inlineStr">
         <is>
-          <t>S35_AG2020</t>
+          <t>S34_NGAEast_Med, S34_NGAEast_SiteAmp, S34_NGAEast_RS24Adj</t>
         </is>
       </c>
       <c r="G285" s="15" t="inlineStr">
         <is>
-          <t>Abrahamson&amp;Gulerce (2020), Global upper Epistemic Model</t>
+          <t>NGA-East 2018 Median Model No. 13 with Stewart et al. (2020) and Hashash et al. (2020) site amplification and Ramos-Sepulveda et al. (2024) adjustments</t>
+        </is>
+      </c>
+      <c r="H285" t="inlineStr">
+        <is>
+          <t>Median only; use with a sigma model (e.g., 7101-7106). VS30 must be 200-3000 m/s</t>
         </is>
       </c>
     </row>
     <row r="286">
-      <c r="B286" s="22" t="n">
-        <v>2392</v>
+      <c r="B286" s="19" t="n">
+        <v>7414</v>
       </c>
       <c r="C286" s="22" t="n">
         <v>25</v>
       </c>
-      <c r="D286" s="22" t="n">
+      <c r="D286" s="23" t="n">
         <v>0.01</v>
       </c>
       <c r="E286" s="23" t="n">
@@ -7341,23 +7428,28 @@
       </c>
       <c r="F286" s="23" t="inlineStr">
         <is>
-          <t>S35_AG2020</t>
+          <t>S34_NGAEast_Med, S34_NGAEast_SiteAmp, S34_NGAEast_RS24Adj</t>
         </is>
       </c>
       <c r="G286" s="15" t="inlineStr">
         <is>
-          <t>Abrahamson&amp;Gulerce (2020), Cascadia with adjustments with Z25=Z25Ref</t>
+          <t>NGA-East 2018 Median Model No. 14 with Stewart et al. (2020) and Hashash et al. (2020) site amplification and Ramos-Sepulveda et al. (2024) adjustments</t>
+        </is>
+      </c>
+      <c r="H286" t="inlineStr">
+        <is>
+          <t>Median only; use with a sigma model (e.g., 7101-7106). VS30 must be 200-3000 m/s</t>
         </is>
       </c>
     </row>
     <row r="287">
-      <c r="B287" s="22" t="n">
-        <v>650</v>
+      <c r="B287" s="19" t="n">
+        <v>7415</v>
       </c>
       <c r="C287" s="22" t="n">
-        <v>23</v>
-      </c>
-      <c r="D287" s="22" t="n">
+        <v>25</v>
+      </c>
+      <c r="D287" s="23" t="n">
         <v>0.01</v>
       </c>
       <c r="E287" s="23" t="n">
@@ -7365,23 +7457,28 @@
       </c>
       <c r="F287" s="23" t="inlineStr">
         <is>
-          <t>S35_KBCG2019</t>
+          <t>S34_NGAEast_Med, S34_NGAEast_SiteAmp, S34_NGAEast_RS24Adj</t>
         </is>
       </c>
       <c r="G287" s="15" t="inlineStr">
         <is>
-          <t>Kuehn et al. (2019), Global</t>
+          <t>NGA-East 2018 Median Model No. 15 with Stewart et al. (2020) and Hashash et al. (2020) site amplification and Ramos-Sepulveda et al. (2024) adjustments</t>
+        </is>
+      </c>
+      <c r="H287" t="inlineStr">
+        <is>
+          <t>Median only; use with a sigma model (e.g., 7101-7106). VS30 must be 200-3000 m/s</t>
         </is>
       </c>
     </row>
     <row r="288">
-      <c r="B288" s="22" t="n">
-        <v>651</v>
+      <c r="B288" s="19" t="n">
+        <v>7416</v>
       </c>
       <c r="C288" s="22" t="n">
-        <v>23</v>
-      </c>
-      <c r="D288" s="22" t="n">
+        <v>25</v>
+      </c>
+      <c r="D288" s="23" t="n">
         <v>0.01</v>
       </c>
       <c r="E288" s="23" t="n">
@@ -7389,23 +7486,28 @@
       </c>
       <c r="F288" s="23" t="inlineStr">
         <is>
-          <t>S35_KBCG2019</t>
+          <t>S34_NGAEast_Med, S34_NGAEast_SiteAmp, S34_NGAEast_RS24Adj</t>
         </is>
       </c>
       <c r="G288" s="15" t="inlineStr">
         <is>
-          <t>Kuehn et al. (2019), Alaska</t>
+          <t>NGA-East 2018 Median Model No. 16 with Stewart et al. (2020) and Hashash et al. (2020) site amplification and Ramos-Sepulveda et al. (2024) adjustments</t>
+        </is>
+      </c>
+      <c r="H288" t="inlineStr">
+        <is>
+          <t>Median only; use with a sigma model (e.g., 7101-7106). VS30 must be 200-3000 m/s</t>
         </is>
       </c>
     </row>
     <row r="289">
-      <c r="B289" s="22" t="n">
-        <v>664</v>
+      <c r="B289" s="19" t="n">
+        <v>7417</v>
       </c>
       <c r="C289" s="22" t="n">
-        <v>23</v>
-      </c>
-      <c r="D289" s="22" t="n">
+        <v>25</v>
+      </c>
+      <c r="D289" s="23" t="n">
         <v>0.01</v>
       </c>
       <c r="E289" s="23" t="n">
@@ -7413,69 +7515,34 @@
       </c>
       <c r="F289" s="23" t="inlineStr">
         <is>
-          <t>S35_KBCG2019</t>
+          <t>S34_NGAEast_Med, S34_NGAEast_SiteAmp, S34_NGAEast_RS24Adj</t>
         </is>
       </c>
       <c r="G289" s="15" t="inlineStr">
         <is>
-          <t>Kuehn et al. (2019), Alaska, mb=8.3</t>
-        </is>
-      </c>
-    </row>
-    <row r="290">
-      <c r="B290" s="22" t="n">
-        <v>665</v>
-      </c>
-      <c r="C290" s="22" t="n">
-        <v>23</v>
-      </c>
-      <c r="D290" s="22" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="E290" s="23" t="n">
-        <v>10</v>
-      </c>
-      <c r="F290" s="23" t="inlineStr">
-        <is>
-          <t>S35_KBCG2019</t>
-        </is>
-      </c>
-      <c r="G290" s="15" t="inlineStr">
-        <is>
-          <t>Kuehn et al. (2019), Alaska, mb=8.9</t>
-        </is>
-      </c>
-    </row>
+          <t>NGA-East 2018 Median Model No. 17 with Stewart et al. (2020) and Hashash et al. (2020) site amplification and Ramos-Sepulveda et al. (2024) adjustments</t>
+        </is>
+      </c>
+      <c r="H289" t="inlineStr">
+        <is>
+          <t>Median only; use with a sigma model (e.g., 7101-7106). VS30 must be 200-3000 m/s</t>
+        </is>
+      </c>
+    </row>
+    <row r="290"/>
     <row r="291">
-      <c r="B291" s="22" t="n">
-        <v>652</v>
-      </c>
-      <c r="C291" s="22" t="n">
-        <v>23</v>
-      </c>
-      <c r="D291" s="22" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="E291" s="23" t="n">
-        <v>10</v>
-      </c>
-      <c r="F291" s="23" t="inlineStr">
-        <is>
-          <t>S35_KBCG2019</t>
-        </is>
-      </c>
-      <c r="G291" s="15" t="inlineStr">
-        <is>
-          <t>Kuehn et al. (2019), Alaska-AluetianIslands</t>
+      <c r="B291" s="26" t="inlineStr">
+        <is>
+          <t>NGA-Subduction</t>
         </is>
       </c>
     </row>
     <row r="292">
       <c r="B292" s="22" t="n">
-        <v>653</v>
+        <v>390</v>
       </c>
       <c r="C292" s="22" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="D292" s="22" t="n">
         <v>0.01</v>
@@ -7485,21 +7552,21 @@
       </c>
       <c r="F292" s="23" t="inlineStr">
         <is>
-          <t>S35_KBCG2019</t>
+          <t>S35_AG2020</t>
         </is>
       </c>
       <c r="G292" s="15" t="inlineStr">
         <is>
-          <t>Kuehn et al. (2019), Cascadia-No-Basin</t>
+          <t>Abrahamson&amp;Gulerce (2020), Alaska without adjustments</t>
         </is>
       </c>
     </row>
     <row r="293">
       <c r="B293" s="22" t="n">
-        <v>662</v>
+        <v>391</v>
       </c>
       <c r="C293" s="22" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="D293" s="22" t="n">
         <v>0.01</v>
@@ -7509,21 +7576,21 @@
       </c>
       <c r="F293" s="23" t="inlineStr">
         <is>
-          <t>S35_KBCG2019</t>
+          <t>S35_AG2020</t>
         </is>
       </c>
       <c r="G293" s="15" t="inlineStr">
         <is>
-          <t>Kuehn et al. (2019), Cascadia-SeattleBasin</t>
+          <t>Abrahamson&amp;Gulerce (2020), Alaska with adjustments</t>
         </is>
       </c>
     </row>
     <row r="294">
       <c r="B294" s="22" t="n">
-        <v>663</v>
+        <v>392</v>
       </c>
       <c r="C294" s="22" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="D294" s="22" t="n">
         <v>0.01</v>
@@ -7533,21 +7600,21 @@
       </c>
       <c r="F294" s="23" t="inlineStr">
         <is>
-          <t>S35_KBCG2019</t>
+          <t>S35_AG2020</t>
         </is>
       </c>
       <c r="G294" s="15" t="inlineStr">
         <is>
-          <t>Kuehn et al. (2019), Cascadia-Non-SeattleBasin</t>
+          <t>Abrahamson&amp;Gulerce (2020), Cascadia with adjustments</t>
         </is>
       </c>
     </row>
     <row r="295">
       <c r="B295" s="22" t="n">
-        <v>654</v>
+        <v>393</v>
       </c>
       <c r="C295" s="22" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="D295" s="22" t="n">
         <v>0.01</v>
@@ -7557,21 +7624,21 @@
       </c>
       <c r="F295" s="23" t="inlineStr">
         <is>
-          <t>S35_KBCG2019</t>
+          <t>S35_AG2020</t>
         </is>
       </c>
       <c r="G295" s="15" t="inlineStr">
         <is>
-          <t>Kuehn et al. (2019), Northern CAM</t>
+          <t>Abrahamson&amp;Gulerce (2020), Central Am/Mexico</t>
         </is>
       </c>
     </row>
     <row r="296">
       <c r="B296" s="22" t="n">
-        <v>655</v>
+        <v>394</v>
       </c>
       <c r="C296" s="22" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="D296" s="22" t="n">
         <v>0.01</v>
@@ -7581,21 +7648,21 @@
       </c>
       <c r="F296" s="23" t="inlineStr">
         <is>
-          <t>S35_KBCG2019</t>
+          <t>S35_AG2020</t>
         </is>
       </c>
       <c r="G296" s="15" t="inlineStr">
         <is>
-          <t>Kuehn et al. (2019), Southern CAM</t>
+          <t>Abrahamson&amp;Gulerce (2020), Japan</t>
         </is>
       </c>
     </row>
     <row r="297">
       <c r="B297" s="22" t="n">
-        <v>656</v>
+        <v>395</v>
       </c>
       <c r="C297" s="22" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="D297" s="22" t="n">
         <v>0.01</v>
@@ -7605,21 +7672,21 @@
       </c>
       <c r="F297" s="23" t="inlineStr">
         <is>
-          <t>S35_KBCG2019</t>
+          <t>S35_AG2020</t>
         </is>
       </c>
       <c r="G297" s="15" t="inlineStr">
         <is>
-          <t>Kuehn et al. (2019), Japan-PacificPlate</t>
+          <t>Abrahamson&amp;Gulerce (2020), New Zealand</t>
         </is>
       </c>
     </row>
     <row r="298">
       <c r="B298" s="22" t="n">
-        <v>657</v>
+        <v>396</v>
       </c>
       <c r="C298" s="22" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="D298" s="22" t="n">
         <v>0.01</v>
@@ -7629,21 +7696,21 @@
       </c>
       <c r="F298" s="23" t="inlineStr">
         <is>
-          <t>S35_KBCG2019</t>
+          <t>S35_AG2020</t>
         </is>
       </c>
       <c r="G298" s="15" t="inlineStr">
         <is>
-          <t>Kuehn et al. (2019), Japan-PhilippinePlate</t>
+          <t>Abrahamson&amp;Gulerce (2020), South America</t>
         </is>
       </c>
     </row>
     <row r="299">
       <c r="B299" s="22" t="n">
-        <v>658</v>
+        <v>397</v>
       </c>
       <c r="C299" s="22" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="D299" s="22" t="n">
         <v>0.01</v>
@@ -7653,21 +7720,21 @@
       </c>
       <c r="F299" s="23" t="inlineStr">
         <is>
-          <t>S35_KBCG2019</t>
+          <t>S35_AG2020</t>
         </is>
       </c>
       <c r="G299" s="15" t="inlineStr">
         <is>
-          <t>Kuehn et al. (2019), Northern SA</t>
+          <t>Abrahamson&amp;Gulerce (2020), Taiwan</t>
         </is>
       </c>
     </row>
     <row r="300">
       <c r="B300" s="22" t="n">
-        <v>659</v>
+        <v>398</v>
       </c>
       <c r="C300" s="22" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="D300" s="22" t="n">
         <v>0.01</v>
@@ -7677,21 +7744,21 @@
       </c>
       <c r="F300" s="23" t="inlineStr">
         <is>
-          <t>S35_KBCG2019</t>
+          <t>S35_AG2020</t>
         </is>
       </c>
       <c r="G300" s="15" t="inlineStr">
         <is>
-          <t>Kuehn et al. (2019), Southern SA</t>
+          <t>Abrahamson&amp;Gulerce (2020), Global</t>
         </is>
       </c>
     </row>
     <row r="301">
       <c r="B301" s="22" t="n">
-        <v>660</v>
+        <v>399</v>
       </c>
       <c r="C301" s="22" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="D301" s="22" t="n">
         <v>0.01</v>
@@ -7701,21 +7768,21 @@
       </c>
       <c r="F301" s="23" t="inlineStr">
         <is>
-          <t>S35_KBCG2019</t>
+          <t>S35_AG2020</t>
         </is>
       </c>
       <c r="G301" s="15" t="inlineStr">
         <is>
-          <t>Kuehn et al. (2019), Taiwan</t>
+          <t>Abrahamson&amp;Gulerce (2020), Cascadia without adjustments</t>
         </is>
       </c>
     </row>
     <row r="302">
       <c r="B302" s="22" t="n">
-        <v>661</v>
+        <v>1398</v>
       </c>
       <c r="C302" s="22" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="D302" s="22" t="n">
         <v>0.01</v>
@@ -7725,21 +7792,21 @@
       </c>
       <c r="F302" s="23" t="inlineStr">
         <is>
-          <t>S35_KBCG2019</t>
+          <t>S35_AG2020</t>
         </is>
       </c>
       <c r="G302" s="15" t="inlineStr">
         <is>
-          <t>Kuehn et al. (2019), New Zealand</t>
+          <t>Abrahamson&amp;Gulerce (2020), Global lower Epistemic Model</t>
         </is>
       </c>
     </row>
     <row r="303">
       <c r="B303" s="22" t="n">
-        <v>610</v>
+        <v>2398</v>
       </c>
       <c r="C303" s="22" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D303" s="22" t="n">
         <v>0.01</v>
@@ -7749,21 +7816,21 @@
       </c>
       <c r="F303" s="23" t="inlineStr">
         <is>
-          <t>S35_PSHAB2019</t>
+          <t>S35_AG2020</t>
         </is>
       </c>
       <c r="G303" s="15" t="inlineStr">
         <is>
-          <t>Parker et al. (2020), Global</t>
+          <t>Abrahamson&amp;Gulerce (2020), Global upper Epistemic Model</t>
         </is>
       </c>
     </row>
     <row r="304">
       <c r="B304" s="22" t="n">
-        <v>611</v>
+        <v>2392</v>
       </c>
       <c r="C304" s="22" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D304" s="22" t="n">
         <v>0.01</v>
@@ -7773,21 +7840,21 @@
       </c>
       <c r="F304" s="23" t="inlineStr">
         <is>
-          <t>S35_PSHAB2019</t>
+          <t>S35_AG2020</t>
         </is>
       </c>
       <c r="G304" s="15" t="inlineStr">
         <is>
-          <t>Parker et al. (2020), Alaska</t>
+          <t>Abrahamson&amp;Gulerce (2020), Cascadia with adjustments with Z25=Z25Ref</t>
         </is>
       </c>
     </row>
     <row r="305">
       <c r="B305" s="22" t="n">
-        <v>612</v>
+        <v>650</v>
       </c>
       <c r="C305" s="22" t="n">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="D305" s="22" t="n">
         <v>0.01</v>
@@ -7797,21 +7864,21 @@
       </c>
       <c r="F305" s="23" t="inlineStr">
         <is>
-          <t>S35_PSHAB2019</t>
+          <t>S35_KBCG2019</t>
         </is>
       </c>
       <c r="G305" s="15" t="inlineStr">
         <is>
-          <t>Parker et al. (2020), Alaska-AleutianIsland</t>
+          <t>Kuehn et al. (2019), Global</t>
         </is>
       </c>
     </row>
     <row r="306">
       <c r="B306" s="22" t="n">
-        <v>613</v>
+        <v>651</v>
       </c>
       <c r="C306" s="22" t="n">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="D306" s="22" t="n">
         <v>0.01</v>
@@ -7821,26 +7888,21 @@
       </c>
       <c r="F306" s="23" t="inlineStr">
         <is>
-          <t>S35_PSHAB2019</t>
+          <t>S35_KBCG2019</t>
         </is>
       </c>
       <c r="G306" s="15" t="inlineStr">
         <is>
-          <t>Parker et al. (2020), Cascadia, Outside Basin</t>
-        </is>
-      </c>
-      <c r="H306" s="15" t="inlineStr">
-        <is>
-          <t>Previous version of the model no longer recommended</t>
+          <t>Kuehn et al. (2019), Alaska</t>
         </is>
       </c>
     </row>
     <row r="307">
       <c r="B307" s="22" t="n">
-        <v>623</v>
+        <v>664</v>
       </c>
       <c r="C307" s="22" t="n">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="D307" s="22" t="n">
         <v>0.01</v>
@@ -7850,21 +7912,21 @@
       </c>
       <c r="F307" s="23" t="inlineStr">
         <is>
-          <t>S35_PSHAB2019</t>
+          <t>S35_KBCG2019</t>
         </is>
       </c>
       <c r="G307" s="15" t="inlineStr">
         <is>
-          <t>Parker et al. (2020), Cascadia with Z25=Z25Ref</t>
+          <t>Kuehn et al. (2019), Alaska, mb=8.3</t>
         </is>
       </c>
     </row>
     <row r="308">
       <c r="B308" s="22" t="n">
-        <v>624</v>
+        <v>665</v>
       </c>
       <c r="C308" s="22" t="n">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="D308" s="22" t="n">
         <v>0.01</v>
@@ -7874,21 +7936,21 @@
       </c>
       <c r="F308" s="23" t="inlineStr">
         <is>
-          <t>S35_PSHAB2019</t>
+          <t>S35_KBCG2019</t>
         </is>
       </c>
       <c r="G308" s="15" t="inlineStr">
         <is>
-          <t>Parker et al. (2020), Cascadia with Z25 value</t>
+          <t>Kuehn et al. (2019), Alaska, mb=8.9</t>
         </is>
       </c>
     </row>
     <row r="309">
       <c r="B309" s="22" t="n">
-        <v>614</v>
+        <v>652</v>
       </c>
       <c r="C309" s="22" t="n">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="D309" s="22" t="n">
         <v>0.01</v>
@@ -7898,26 +7960,21 @@
       </c>
       <c r="F309" s="23" t="inlineStr">
         <is>
-          <t>S35_PSHAB2019</t>
+          <t>S35_KBCG2019</t>
         </is>
       </c>
       <c r="G309" s="15" t="inlineStr">
         <is>
-          <t>Parker et al. (2020), Cascadia, Seattle Basin</t>
-        </is>
-      </c>
-      <c r="H309" s="15" t="inlineStr">
-        <is>
-          <t>Previous version of the model no longer recommended</t>
+          <t>Kuehn et al. (2019), Alaska-AluetianIslands</t>
         </is>
       </c>
     </row>
     <row r="310">
       <c r="B310" s="22" t="n">
-        <v>615</v>
+        <v>653</v>
       </c>
       <c r="C310" s="22" t="n">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="D310" s="22" t="n">
         <v>0.01</v>
@@ -7927,26 +7984,21 @@
       </c>
       <c r="F310" s="23" t="inlineStr">
         <is>
-          <t>S35_PSHAB2019</t>
+          <t>S35_KBCG2019</t>
         </is>
       </c>
       <c r="G310" s="15" t="inlineStr">
         <is>
-          <t>Parker et al. (2020), Cascadia, Other PNW Basin</t>
-        </is>
-      </c>
-      <c r="H310" s="15" t="inlineStr">
-        <is>
-          <t>Previous version of the model no longer recommended</t>
+          <t>Kuehn et al. (2019), Cascadia-No-Basin</t>
         </is>
       </c>
     </row>
     <row r="311">
       <c r="B311" s="22" t="n">
-        <v>616</v>
+        <v>662</v>
       </c>
       <c r="C311" s="22" t="n">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="D311" s="22" t="n">
         <v>0.01</v>
@@ -7956,21 +8008,21 @@
       </c>
       <c r="F311" s="23" t="inlineStr">
         <is>
-          <t>S35_PSHAB2019</t>
+          <t>S35_KBCG2019</t>
         </is>
       </c>
       <c r="G311" s="15" t="inlineStr">
         <is>
-          <t>Parker et al. (2020), Northern-CAM</t>
+          <t>Kuehn et al. (2019), Cascadia-SeattleBasin</t>
         </is>
       </c>
     </row>
     <row r="312">
       <c r="B312" s="22" t="n">
-        <v>617</v>
+        <v>663</v>
       </c>
       <c r="C312" s="22" t="n">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="D312" s="22" t="n">
         <v>0.01</v>
@@ -7980,21 +8032,21 @@
       </c>
       <c r="F312" s="23" t="inlineStr">
         <is>
-          <t>S35_PSHAB2019</t>
+          <t>S35_KBCG2019</t>
         </is>
       </c>
       <c r="G312" s="15" t="inlineStr">
         <is>
-          <t>Parker et al. (2020), Southern-CAM</t>
+          <t>Kuehn et al. (2019), Cascadia-Non-SeattleBasin</t>
         </is>
       </c>
     </row>
     <row r="313">
       <c r="B313" s="22" t="n">
-        <v>618</v>
+        <v>654</v>
       </c>
       <c r="C313" s="22" t="n">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="D313" s="22" t="n">
         <v>0.01</v>
@@ -8004,21 +8056,21 @@
       </c>
       <c r="F313" s="23" t="inlineStr">
         <is>
-          <t>S35_PSHAB2019</t>
+          <t>S35_KBCG2019</t>
         </is>
       </c>
       <c r="G313" s="15" t="inlineStr">
         <is>
-          <t>Parker et al. (2020), Japan-PacificPlate with Z25 value</t>
+          <t>Kuehn et al. (2019), Northern CAM</t>
         </is>
       </c>
     </row>
     <row r="314">
       <c r="B314" s="22" t="n">
-        <v>625</v>
+        <v>655</v>
       </c>
       <c r="C314" s="22" t="n">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="D314" s="22" t="n">
         <v>0.01</v>
@@ -8028,26 +8080,21 @@
       </c>
       <c r="F314" s="23" t="inlineStr">
         <is>
-          <t>S35_PSHAB2019</t>
+          <t>S35_KBCG2019</t>
         </is>
       </c>
       <c r="G314" s="15" t="inlineStr">
         <is>
-          <t>Parker et al. (2020), Japan-PacificPlate with Z25=Z25Ref</t>
-        </is>
-      </c>
-      <c r="H314" s="15" t="inlineStr">
-        <is>
-          <t>No basin effects</t>
+          <t>Kuehn et al. (2019), Southern CAM</t>
         </is>
       </c>
     </row>
     <row r="315">
       <c r="B315" s="22" t="n">
-        <v>619</v>
+        <v>656</v>
       </c>
       <c r="C315" s="22" t="n">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="D315" s="22" t="n">
         <v>0.01</v>
@@ -8057,21 +8104,21 @@
       </c>
       <c r="F315" s="23" t="inlineStr">
         <is>
-          <t>S35_PSHAB2019</t>
+          <t>S35_KBCG2019</t>
         </is>
       </c>
       <c r="G315" s="15" t="inlineStr">
         <is>
-          <t>Parker et al. (2020), Japan-PhilippinePlate with Z25 value</t>
+          <t>Kuehn et al. (2019), Japan-PacificPlate</t>
         </is>
       </c>
     </row>
     <row r="316">
       <c r="B316" s="22" t="n">
-        <v>626</v>
+        <v>657</v>
       </c>
       <c r="C316" s="22" t="n">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="D316" s="22" t="n">
         <v>0.01</v>
@@ -8081,26 +8128,21 @@
       </c>
       <c r="F316" s="23" t="inlineStr">
         <is>
-          <t>S35_PSHAB2019</t>
+          <t>S35_KBCG2019</t>
         </is>
       </c>
       <c r="G316" s="15" t="inlineStr">
         <is>
-          <t>Parker et al. (2020), Japan-PhilippinePlate with Z25=Z25Ref</t>
-        </is>
-      </c>
-      <c r="H316" s="15" t="inlineStr">
-        <is>
-          <t>No basin effects</t>
+          <t>Kuehn et al. (2019), Japan-PhilippinePlate</t>
         </is>
       </c>
     </row>
     <row r="317">
       <c r="B317" s="22" t="n">
-        <v>620</v>
+        <v>658</v>
       </c>
       <c r="C317" s="22" t="n">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="D317" s="22" t="n">
         <v>0.01</v>
@@ -8110,21 +8152,21 @@
       </c>
       <c r="F317" s="23" t="inlineStr">
         <is>
-          <t>S35_PSHAB2019</t>
+          <t>S35_KBCG2019</t>
         </is>
       </c>
       <c r="G317" s="15" t="inlineStr">
         <is>
-          <t>Parker et al. (2020), Northern-SA</t>
+          <t>Kuehn et al. (2019), Northern SA</t>
         </is>
       </c>
     </row>
     <row r="318">
       <c r="B318" s="22" t="n">
-        <v>621</v>
+        <v>659</v>
       </c>
       <c r="C318" s="22" t="n">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="D318" s="22" t="n">
         <v>0.01</v>
@@ -8134,21 +8176,21 @@
       </c>
       <c r="F318" s="23" t="inlineStr">
         <is>
-          <t>S35_PSHAB2019</t>
+          <t>S35_KBCG2019</t>
         </is>
       </c>
       <c r="G318" s="15" t="inlineStr">
         <is>
-          <t>Parker et al. (2020), Southern-SA</t>
+          <t>Kuehn et al. (2019), Southern SA</t>
         </is>
       </c>
     </row>
     <row r="319">
       <c r="B319" s="22" t="n">
-        <v>622</v>
+        <v>660</v>
       </c>
       <c r="C319" s="22" t="n">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="D319" s="22" t="n">
         <v>0.01</v>
@@ -8158,18 +8200,18 @@
       </c>
       <c r="F319" s="23" t="inlineStr">
         <is>
-          <t>S35_PSHAB2019</t>
+          <t>S35_KBCG2019</t>
         </is>
       </c>
       <c r="G319" s="15" t="inlineStr">
         <is>
-          <t>Parker et al. (2020), Taiwan-East</t>
+          <t>Kuehn et al. (2019), Taiwan</t>
         </is>
       </c>
     </row>
     <row r="320">
       <c r="B320" s="22" t="n">
-        <v>675</v>
+        <v>661</v>
       </c>
       <c r="C320" s="22" t="n">
         <v>23</v>
@@ -8182,287 +8224,745 @@
       </c>
       <c r="F320" s="23" t="inlineStr">
         <is>
-          <t>S35_SMK2020</t>
+          <t>S35_KBCG2019</t>
         </is>
       </c>
       <c r="G320" s="15" t="inlineStr">
         <is>
-          <t>Si, Midorikawa, and Kishida (2020), Japan-No Basin</t>
+          <t>Kuehn et al. (2019), New Zealand</t>
         </is>
       </c>
     </row>
     <row r="321">
       <c r="B321" s="22" t="n">
+        <v>610</v>
+      </c>
+      <c r="C321" s="22" t="n">
+        <v>26</v>
+      </c>
+      <c r="D321" s="22" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="E321" s="23" t="n">
+        <v>10</v>
+      </c>
+      <c r="F321" s="23" t="inlineStr">
+        <is>
+          <t>S35_PSHAB2019</t>
+        </is>
+      </c>
+      <c r="G321" s="15" t="inlineStr">
+        <is>
+          <t>Parker et al. (2020), Global</t>
+        </is>
+      </c>
+    </row>
+    <row r="322">
+      <c r="B322" s="22" t="n">
+        <v>611</v>
+      </c>
+      <c r="C322" s="22" t="n">
+        <v>26</v>
+      </c>
+      <c r="D322" s="22" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="E322" s="23" t="n">
+        <v>10</v>
+      </c>
+      <c r="F322" s="23" t="inlineStr">
+        <is>
+          <t>S35_PSHAB2019</t>
+        </is>
+      </c>
+      <c r="G322" s="15" t="inlineStr">
+        <is>
+          <t>Parker et al. (2020), Alaska</t>
+        </is>
+      </c>
+    </row>
+    <row r="323">
+      <c r="B323" s="22" t="n">
+        <v>612</v>
+      </c>
+      <c r="C323" s="22" t="n">
+        <v>26</v>
+      </c>
+      <c r="D323" s="22" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="E323" s="23" t="n">
+        <v>10</v>
+      </c>
+      <c r="F323" s="23" t="inlineStr">
+        <is>
+          <t>S35_PSHAB2019</t>
+        </is>
+      </c>
+      <c r="G323" s="15" t="inlineStr">
+        <is>
+          <t>Parker et al. (2020), Alaska-AleutianIsland</t>
+        </is>
+      </c>
+    </row>
+    <row r="324">
+      <c r="B324" s="22" t="n">
+        <v>613</v>
+      </c>
+      <c r="C324" s="22" t="n">
+        <v>26</v>
+      </c>
+      <c r="D324" s="22" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="E324" s="23" t="n">
+        <v>10</v>
+      </c>
+      <c r="F324" s="23" t="inlineStr">
+        <is>
+          <t>S35_PSHAB2019</t>
+        </is>
+      </c>
+      <c r="G324" s="15" t="inlineStr">
+        <is>
+          <t>Parker et al. (2020), Cascadia, Outside Basin</t>
+        </is>
+      </c>
+      <c r="H324" s="15" t="inlineStr">
+        <is>
+          <t>Previous version of the model no longer recommended</t>
+        </is>
+      </c>
+    </row>
+    <row r="325">
+      <c r="B325" s="22" t="n">
+        <v>623</v>
+      </c>
+      <c r="C325" s="22" t="n">
+        <v>26</v>
+      </c>
+      <c r="D325" s="22" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="E325" s="23" t="n">
+        <v>10</v>
+      </c>
+      <c r="F325" s="23" t="inlineStr">
+        <is>
+          <t>S35_PSHAB2019</t>
+        </is>
+      </c>
+      <c r="G325" s="15" t="inlineStr">
+        <is>
+          <t>Parker et al. (2020), Cascadia with Z25=Z25Ref</t>
+        </is>
+      </c>
+    </row>
+    <row r="326">
+      <c r="B326" s="22" t="n">
+        <v>624</v>
+      </c>
+      <c r="C326" s="22" t="n">
+        <v>26</v>
+      </c>
+      <c r="D326" s="22" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="E326" s="23" t="n">
+        <v>10</v>
+      </c>
+      <c r="F326" s="23" t="inlineStr">
+        <is>
+          <t>S35_PSHAB2019</t>
+        </is>
+      </c>
+      <c r="G326" s="15" t="inlineStr">
+        <is>
+          <t>Parker et al. (2020), Cascadia with Z25 value</t>
+        </is>
+      </c>
+    </row>
+    <row r="327">
+      <c r="B327" s="22" t="n">
+        <v>614</v>
+      </c>
+      <c r="C327" s="22" t="n">
+        <v>26</v>
+      </c>
+      <c r="D327" s="22" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="E327" s="23" t="n">
+        <v>10</v>
+      </c>
+      <c r="F327" s="23" t="inlineStr">
+        <is>
+          <t>S35_PSHAB2019</t>
+        </is>
+      </c>
+      <c r="G327" s="15" t="inlineStr">
+        <is>
+          <t>Parker et al. (2020), Cascadia, Seattle Basin</t>
+        </is>
+      </c>
+      <c r="H327" s="15" t="inlineStr">
+        <is>
+          <t>Previous version of the model no longer recommended</t>
+        </is>
+      </c>
+    </row>
+    <row r="328">
+      <c r="B328" s="22" t="n">
+        <v>615</v>
+      </c>
+      <c r="C328" s="22" t="n">
+        <v>26</v>
+      </c>
+      <c r="D328" s="22" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="E328" s="23" t="n">
+        <v>10</v>
+      </c>
+      <c r="F328" s="23" t="inlineStr">
+        <is>
+          <t>S35_PSHAB2019</t>
+        </is>
+      </c>
+      <c r="G328" s="15" t="inlineStr">
+        <is>
+          <t>Parker et al. (2020), Cascadia, Other PNW Basin</t>
+        </is>
+      </c>
+      <c r="H328" s="15" t="inlineStr">
+        <is>
+          <t>Previous version of the model no longer recommended</t>
+        </is>
+      </c>
+    </row>
+    <row r="329">
+      <c r="B329" s="22" t="n">
+        <v>616</v>
+      </c>
+      <c r="C329" s="22" t="n">
+        <v>26</v>
+      </c>
+      <c r="D329" s="22" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="E329" s="23" t="n">
+        <v>10</v>
+      </c>
+      <c r="F329" s="23" t="inlineStr">
+        <is>
+          <t>S35_PSHAB2019</t>
+        </is>
+      </c>
+      <c r="G329" s="15" t="inlineStr">
+        <is>
+          <t>Parker et al. (2020), Northern-CAM</t>
+        </is>
+      </c>
+    </row>
+    <row r="330">
+      <c r="B330" s="22" t="n">
+        <v>617</v>
+      </c>
+      <c r="C330" s="22" t="n">
+        <v>26</v>
+      </c>
+      <c r="D330" s="22" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="E330" s="23" t="n">
+        <v>10</v>
+      </c>
+      <c r="F330" s="23" t="inlineStr">
+        <is>
+          <t>S35_PSHAB2019</t>
+        </is>
+      </c>
+      <c r="G330" s="15" t="inlineStr">
+        <is>
+          <t>Parker et al. (2020), Southern-CAM</t>
+        </is>
+      </c>
+    </row>
+    <row r="331">
+      <c r="B331" s="22" t="n">
+        <v>618</v>
+      </c>
+      <c r="C331" s="22" t="n">
+        <v>26</v>
+      </c>
+      <c r="D331" s="22" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="E331" s="23" t="n">
+        <v>10</v>
+      </c>
+      <c r="F331" s="23" t="inlineStr">
+        <is>
+          <t>S35_PSHAB2019</t>
+        </is>
+      </c>
+      <c r="G331" s="15" t="inlineStr">
+        <is>
+          <t>Parker et al. (2020), Japan-PacificPlate with Z25 value</t>
+        </is>
+      </c>
+    </row>
+    <row r="332">
+      <c r="B332" s="22" t="n">
+        <v>625</v>
+      </c>
+      <c r="C332" s="22" t="n">
+        <v>26</v>
+      </c>
+      <c r="D332" s="22" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="E332" s="23" t="n">
+        <v>10</v>
+      </c>
+      <c r="F332" s="23" t="inlineStr">
+        <is>
+          <t>S35_PSHAB2019</t>
+        </is>
+      </c>
+      <c r="G332" s="15" t="inlineStr">
+        <is>
+          <t>Parker et al. (2020), Japan-PacificPlate with Z25=Z25Ref</t>
+        </is>
+      </c>
+      <c r="H332" s="15" t="inlineStr">
+        <is>
+          <t>No basin effects</t>
+        </is>
+      </c>
+    </row>
+    <row r="333">
+      <c r="B333" s="22" t="n">
+        <v>619</v>
+      </c>
+      <c r="C333" s="22" t="n">
+        <v>26</v>
+      </c>
+      <c r="D333" s="22" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="E333" s="23" t="n">
+        <v>10</v>
+      </c>
+      <c r="F333" s="23" t="inlineStr">
+        <is>
+          <t>S35_PSHAB2019</t>
+        </is>
+      </c>
+      <c r="G333" s="15" t="inlineStr">
+        <is>
+          <t>Parker et al. (2020), Japan-PhilippinePlate with Z25 value</t>
+        </is>
+      </c>
+    </row>
+    <row r="334">
+      <c r="B334" s="22" t="n">
+        <v>626</v>
+      </c>
+      <c r="C334" s="22" t="n">
+        <v>26</v>
+      </c>
+      <c r="D334" s="22" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="E334" s="23" t="n">
+        <v>10</v>
+      </c>
+      <c r="F334" s="23" t="inlineStr">
+        <is>
+          <t>S35_PSHAB2019</t>
+        </is>
+      </c>
+      <c r="G334" s="15" t="inlineStr">
+        <is>
+          <t>Parker et al. (2020), Japan-PhilippinePlate with Z25=Z25Ref</t>
+        </is>
+      </c>
+      <c r="H334" s="15" t="inlineStr">
+        <is>
+          <t>No basin effects</t>
+        </is>
+      </c>
+    </row>
+    <row r="335">
+      <c r="B335" s="22" t="n">
+        <v>620</v>
+      </c>
+      <c r="C335" s="22" t="n">
+        <v>26</v>
+      </c>
+      <c r="D335" s="22" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="E335" s="23" t="n">
+        <v>10</v>
+      </c>
+      <c r="F335" s="23" t="inlineStr">
+        <is>
+          <t>S35_PSHAB2019</t>
+        </is>
+      </c>
+      <c r="G335" s="15" t="inlineStr">
+        <is>
+          <t>Parker et al. (2020), Northern-SA</t>
+        </is>
+      </c>
+    </row>
+    <row r="336">
+      <c r="B336" s="22" t="n">
+        <v>621</v>
+      </c>
+      <c r="C336" s="22" t="n">
+        <v>26</v>
+      </c>
+      <c r="D336" s="22" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="E336" s="23" t="n">
+        <v>10</v>
+      </c>
+      <c r="F336" s="23" t="inlineStr">
+        <is>
+          <t>S35_PSHAB2019</t>
+        </is>
+      </c>
+      <c r="G336" s="15" t="inlineStr">
+        <is>
+          <t>Parker et al. (2020), Southern-SA</t>
+        </is>
+      </c>
+    </row>
+    <row r="337">
+      <c r="B337" s="22" t="n">
+        <v>622</v>
+      </c>
+      <c r="C337" s="22" t="n">
+        <v>26</v>
+      </c>
+      <c r="D337" s="22" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="E337" s="23" t="n">
+        <v>10</v>
+      </c>
+      <c r="F337" s="23" t="inlineStr">
+        <is>
+          <t>S35_PSHAB2019</t>
+        </is>
+      </c>
+      <c r="G337" s="15" t="inlineStr">
+        <is>
+          <t>Parker et al. (2020), Taiwan-East</t>
+        </is>
+      </c>
+    </row>
+    <row r="338">
+      <c r="B338" s="22" t="n">
+        <v>675</v>
+      </c>
+      <c r="C338" s="22" t="n">
+        <v>23</v>
+      </c>
+      <c r="D338" s="22" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="E338" s="23" t="n">
+        <v>10</v>
+      </c>
+      <c r="F338" s="23" t="inlineStr">
+        <is>
+          <t>S35_SMK2020</t>
+        </is>
+      </c>
+      <c r="G338" s="15" t="inlineStr">
+        <is>
+          <t>Si, Midorikawa, and Kishida (2020), Japan-No Basin</t>
+        </is>
+      </c>
+    </row>
+    <row r="339">
+      <c r="B339" s="22" t="n">
         <v>676</v>
       </c>
-      <c r="C321" s="22" t="n">
+      <c r="C339" s="22" t="n">
         <v>23</v>
       </c>
-      <c r="D321" s="22" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="E321" s="23" t="n">
-        <v>10</v>
-      </c>
-      <c r="F321" s="23" t="inlineStr">
+      <c r="D339" s="22" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="E339" s="23" t="n">
+        <v>10</v>
+      </c>
+      <c r="F339" s="23" t="inlineStr">
         <is>
           <t>S35_SMK2020</t>
         </is>
       </c>
-      <c r="G321" s="15" t="inlineStr">
+      <c r="G339" s="15" t="inlineStr">
         <is>
           <t>Si, Midorikawa, and Kishida (2020), Japan with Basin</t>
         </is>
       </c>
     </row>
-    <row r="323">
-      <c r="B323" s="26" t="inlineStr">
+    <row r="340"/>
+    <row r="341">
+      <c r="B341" s="26" t="inlineStr">
         <is>
           <t>Stable Continental Region Ground Motion Models (Australia, Brazil, Europe)</t>
         </is>
       </c>
     </row>
-    <row r="324">
-      <c r="B324" s="19" t="n">
+    <row r="342">
+      <c r="B342" s="19" t="n">
         <v>1234</v>
       </c>
-      <c r="C324" s="22" t="n">
+      <c r="C342" s="22" t="n">
         <v>22</v>
       </c>
-      <c r="D324" s="23" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="E324" s="23" t="n">
-        <v>10</v>
-      </c>
-      <c r="F324" s="23" t="inlineStr">
+      <c r="D342" s="23" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="E342" s="23" t="n">
+        <v>10</v>
+      </c>
+      <c r="F342" s="23" t="inlineStr">
         <is>
           <t>S02_Somerville_2009_Craton</t>
         </is>
       </c>
-      <c r="G324" s="15" t="inlineStr">
+      <c r="G342" s="15" t="inlineStr">
         <is>
           <t>Somerville et al. (2009), Australia, Cratonic (Yilgarn Craton model)</t>
         </is>
       </c>
     </row>
-    <row r="325">
-      <c r="B325" s="19" t="n">
+    <row r="343">
+      <c r="B343" s="19" t="n">
         <v>1235</v>
       </c>
-      <c r="C325" s="22" t="n">
+      <c r="C343" s="22" t="n">
         <v>22</v>
       </c>
-      <c r="D325" s="23" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="E325" s="23" t="n">
-        <v>10</v>
-      </c>
-      <c r="F325" s="23" t="inlineStr">
+      <c r="D343" s="23" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="E343" s="23" t="n">
+        <v>10</v>
+      </c>
+      <c r="F343" s="23" t="inlineStr">
         <is>
           <t>S02_Somerville_2009_NonCraton</t>
         </is>
       </c>
-      <c r="G325" s="15" t="inlineStr">
+      <c r="G343" s="15" t="inlineStr">
         <is>
           <t>Somerville et al. (2009), Australia, Non-Cratonic</t>
         </is>
       </c>
     </row>
-    <row r="326">
-      <c r="B326" s="19" t="n">
+    <row r="344">
+      <c r="B344" s="19" t="n">
         <v>1236</v>
       </c>
-      <c r="C326" s="22" t="n">
+      <c r="C344" s="22" t="n">
         <v>18</v>
       </c>
-      <c r="D326" s="23" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="E326" s="23" t="n">
+      <c r="D344" s="23" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="E344" s="23" t="n">
         <v>4</v>
       </c>
-      <c r="F326" s="23" t="inlineStr">
+      <c r="F344" s="23" t="inlineStr">
         <is>
           <t>S02_Allen_2012</t>
         </is>
       </c>
-      <c r="G326" s="15" t="inlineStr">
+      <c r="G344" s="15" t="inlineStr">
         <is>
           <t>Allen (2012), Southeastern Australia</t>
         </is>
       </c>
-      <c r="H326" t="inlineStr">
+      <c r="H344" t="inlineStr">
         <is>
           <t>Shallow or deep coefficients selected by hypocentral depth (10 km)</t>
         </is>
       </c>
     </row>
-    <row r="327">
-      <c r="B327" s="19" t="n">
+    <row r="345">
+      <c r="B345" s="19" t="n">
         <v>1237</v>
       </c>
-      <c r="C327" s="22" t="n">
+      <c r="C345" s="22" t="n">
         <v>20</v>
       </c>
-      <c r="D327" s="23" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="E327" s="23" t="n">
+      <c r="D345" s="23" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="E345" s="23" t="n">
         <v>3</v>
       </c>
-      <c r="F327" s="23" t="inlineStr">
+      <c r="F345" s="23" t="inlineStr">
         <is>
           <t>S02_Drouet_2015_Brazil</t>
         </is>
       </c>
-      <c r="G327" s="15" t="inlineStr">
+      <c r="G345" s="15" t="inlineStr">
         <is>
           <t>Drouet (2015), Brazil</t>
         </is>
       </c>
     </row>
-    <row r="328">
-      <c r="B328" s="19" t="n">
+    <row r="346">
+      <c r="B346" s="19" t="n">
         <v>1238</v>
       </c>
-      <c r="C328" s="22" t="n">
+      <c r="C346" s="22" t="n">
         <v>23</v>
       </c>
-      <c r="D328" s="23" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="E328" s="23" t="n">
-        <v>10</v>
-      </c>
-      <c r="F328" s="23" t="inlineStr">
+      <c r="D346" s="23" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="E346" s="23" t="n">
+        <v>10</v>
+      </c>
+      <c r="F346" s="23" t="inlineStr">
         <is>
           <t>S02_ESHM2020_Craton</t>
         </is>
       </c>
-      <c r="G328" s="15" t="inlineStr">
+      <c r="G346" s="15" t="inlineStr">
         <is>
           <t>Weatherill and Cotton (2020), ESHM20 Craton (VS30 = 3000 m/s)</t>
         </is>
       </c>
-      <c r="H328" t="inlineStr">
+      <c r="H346" t="inlineStr">
         <is>
           <t>Median only; use with a sigma model (e.g., 7101-7106)</t>
         </is>
       </c>
     </row>
-    <row r="329">
-      <c r="B329" s="19" t="n">
+    <row r="347">
+      <c r="B347" s="19" t="n">
         <v>1239</v>
       </c>
-      <c r="C329" s="22" t="n">
+      <c r="C347" s="22" t="n">
         <v>23</v>
       </c>
-      <c r="D329" s="23" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="E329" s="23" t="n">
-        <v>10</v>
-      </c>
-      <c r="F329" s="23" t="inlineStr">
+      <c r="D347" s="23" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="E347" s="23" t="n">
+        <v>10</v>
+      </c>
+      <c r="F347" s="23" t="inlineStr">
         <is>
           <t>S02_ESHM2020_Craton, S34_NGAEast_SiteAmp</t>
         </is>
       </c>
-      <c r="G329" s="15" t="inlineStr">
+      <c r="G347" s="15" t="inlineStr">
         <is>
           <t>Weatherill and Cotton (2020), ESHM20 Craton with Stewart et al. (2020) and Hashash et al. (2020) site amplification</t>
         </is>
       </c>
-      <c r="H329" t="inlineStr">
+      <c r="H347" t="inlineStr">
         <is>
           <t>Median only; use with a sigma model (e.g., 7101-7106). VS30 must be 200-3000 m/s</t>
         </is>
       </c>
     </row>
-    <row r="330">
-      <c r="B330" s="19" t="n">
+    <row r="348">
+      <c r="B348" s="19" t="n">
         <v>1240</v>
       </c>
-      <c r="C330" s="22" t="n">
+      <c r="C348" s="22" t="n">
         <v>20</v>
       </c>
-      <c r="D330" s="23" t="n">
+      <c r="D348" s="23" t="n">
         <v>0.1</v>
       </c>
-      <c r="E330" s="23" t="n">
-        <v>10</v>
-      </c>
-      <c r="F330" s="23" t="inlineStr">
+      <c r="E348" s="23" t="n">
+        <v>10</v>
+      </c>
+      <c r="F348" s="23" t="inlineStr">
         <is>
           <t>S02_Allen_2022</t>
         </is>
       </c>
-      <c r="G330" s="15" t="inlineStr">
+      <c r="G348" s="15" t="inlineStr">
         <is>
           <t>Allen (2022), Far-field North Australian Craton</t>
         </is>
       </c>
-      <c r="H330" t="inlineStr">
+      <c r="H348" t="inlineStr">
         <is>
           <t>VS30 must be 220-800 m/s</t>
         </is>
       </c>
     </row>
-    <row r="331">
-      <c r="B331" s="19" t="n">
+    <row r="349">
+      <c r="B349" s="19" t="n">
         <v>1241</v>
       </c>
-      <c r="C331" s="22" t="n">
+      <c r="C349" s="22" t="n">
         <v>63</v>
       </c>
-      <c r="D331" s="23" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="E331" s="23" t="n">
-        <v>10</v>
-      </c>
-      <c r="F331" s="23" t="inlineStr">
+      <c r="D349" s="23" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="E349" s="23" t="n">
+        <v>10</v>
+      </c>
+      <c r="F349" s="23" t="inlineStr">
         <is>
           <t>S02_BS_2024</t>
         </is>
       </c>
-      <c r="G331" s="15" t="inlineStr">
+      <c r="G349" s="15" t="inlineStr">
         <is>
           <t>Bayless and Somerville (2024), Australia, Cratonic</t>
         </is>
       </c>
-      <c r="H331" t="inlineStr">
+      <c r="H349" t="inlineStr">
         <is>
           <t>Z1.0 scaling not applied</t>
         </is>
       </c>
     </row>
-    <row r="332">
-      <c r="B332" s="19" t="n">
+    <row r="350">
+      <c r="B350" s="19" t="n">
         <v>1242</v>
       </c>
-      <c r="C332" s="22" t="n">
+      <c r="C350" s="22" t="n">
         <v>63</v>
       </c>
-      <c r="D332" s="23" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="E332" s="23" t="n">
-        <v>10</v>
-      </c>
-      <c r="F332" s="23" t="inlineStr">
+      <c r="D350" s="23" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="E350" s="23" t="n">
+        <v>10</v>
+      </c>
+      <c r="F350" s="23" t="inlineStr">
         <is>
           <t>S02_BS_2024</t>
         </is>
       </c>
-      <c r="G332" s="15" t="inlineStr">
+      <c r="G350" s="15" t="inlineStr">
         <is>
           <t>Bayless and Somerville (2024), Australia, Non-Cratonic</t>
         </is>
       </c>
-      <c r="H332" t="inlineStr">
+      <c r="H350" t="inlineStr">
         <is>
           <t>Z1.0 scaling not applied</t>
         </is>
@@ -8483,7 +8983,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I232"/>
+  <dimension ref="B1:I232"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="10.75" defaultRowHeight="15.5"/>
   <cols>
     <col width="9.25" customWidth="1" style="15" min="1" max="1"/>
@@ -8503,7 +9003,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="B3" s="1" t="inlineStr">
         <is>

</xml_diff>